<commit_message>
fix: corrige le lien de la maquette et met à jour les prénoms de l'équipe (Flo, Michou, Krys)
</commit_message>
<xml_diff>
--- a/docs/Kernel_Repartition_Taches.xlsx
+++ b/docs/Kernel_Repartition_Taches.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -54,13 +54,13 @@
     <t xml:space="preserve">Florette</t>
   </si>
   <si>
-    <t xml:space="preserve">Coéquipier 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coéquipier 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coéquipier 4</t>
+    <t xml:space="preserve">Flo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Michou</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Krys</t>
   </si>
   <si>
     <t xml:space="preserve">Légende des statuts</t>
@@ -583,44 +583,48 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -700,7 +704,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -963,97 +967,97 @@
   <dimension ref="B2:B23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="95"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+    <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="5" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="5" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="6" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="5" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="5" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="6" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="7" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B20" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="8" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="8" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B22" s="9" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="9" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B23" s="10" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1076,794 +1080,794 @@
   <dimension ref="A1:I27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="G1" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="H1" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="I1" s="11" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="11" t="n">
+      <c r="A2" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="14" t="s">
+      <c r="E2" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="F2" s="14" t="s">
+      <c r="F2" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11" t="n">
+      <c r="G2" s="12"/>
+      <c r="H2" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="I2" s="15" t="s">
+      <c r="I2" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="16" t="n">
+      <c r="A3" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="D3" s="17" t="s">
+      <c r="D3" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="G3" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="H3" s="16" t="n">
+      <c r="H3" s="17" t="n">
         <v>0.5</v>
       </c>
-      <c r="I3" s="15" t="s">
+      <c r="I3" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="n">
+      <c r="A4" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="E4" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="G4" s="11" t="s">
+      <c r="G4" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="H4" s="11" t="n">
+      <c r="H4" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="I4" s="15" t="s">
+      <c r="I4" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="16" t="n">
+      <c r="A5" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="17" t="s">
+      <c r="D5" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="18" t="s">
+      <c r="E5" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="F5" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="G5" s="16" t="s">
+      <c r="G5" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="H5" s="16" t="n">
+      <c r="H5" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="I5" s="15" t="s">
+      <c r="I5" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="n">
+      <c r="A6" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="14" t="s">
+      <c r="E6" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="G6" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="H6" s="11" t="n">
+      <c r="H6" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="I6" s="15" t="s">
+      <c r="I6" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="16" t="n">
+      <c r="A7" s="17" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="16" t="s">
+      <c r="B7" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="17" t="s">
+      <c r="D7" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="E7" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="F7" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="G7" s="16" t="s">
+      <c r="G7" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="H7" s="16" t="n">
+      <c r="H7" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="I7" s="15" t="s">
+      <c r="I7" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="n">
+      <c r="A8" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="G8" s="11" t="s">
+      <c r="G8" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="H8" s="11" t="n">
+      <c r="H8" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="I8" s="15" t="s">
+      <c r="I8" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="16" t="n">
+      <c r="A9" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="16" t="s">
+      <c r="B9" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="D9" s="17" t="s">
+      <c r="D9" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="18" t="s">
+      <c r="E9" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="F9" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="G9" s="16" t="s">
+      <c r="G9" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="H9" s="16" t="n">
+      <c r="H9" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="I9" s="15" t="s">
+      <c r="I9" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="n">
+      <c r="A10" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="E10" s="14" t="s">
+      <c r="E10" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="F10" s="14" t="s">
+      <c r="F10" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="G10" s="11" t="s">
+      <c r="G10" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="H10" s="11" t="n">
+      <c r="H10" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="I10" s="15" t="s">
+      <c r="I10" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="16" t="n">
+      <c r="A11" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="D11" s="17" t="s">
+      <c r="D11" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="E11" s="18" t="s">
+      <c r="E11" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="F11" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="G11" s="16" t="s">
+      <c r="G11" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="H11" s="16" t="n">
+      <c r="H11" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="I11" s="15" t="s">
+      <c r="I11" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="n">
+      <c r="A12" s="12" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="C12" s="19" t="s">
+      <c r="C12" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="14" t="s">
+      <c r="E12" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="F12" s="14" t="s">
+      <c r="F12" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="G12" s="11" t="s">
+      <c r="G12" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="H12" s="11" t="n">
+      <c r="H12" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="I12" s="15" t="s">
+      <c r="I12" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="16" t="n">
+      <c r="A13" s="17" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="16" t="s">
+      <c r="B13" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="C13" s="20" t="s">
+      <c r="C13" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="D13" s="17" t="s">
+      <c r="D13" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="E13" s="18" t="s">
+      <c r="E13" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="F13" s="18" t="s">
+      <c r="F13" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="G13" s="16" t="s">
+      <c r="G13" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="H13" s="16" t="n">
+      <c r="H13" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="I13" s="15" t="s">
+      <c r="I13" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="n">
+      <c r="A14" s="12" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="C14" s="20" t="s">
+      <c r="C14" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="D14" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="E14" s="14" t="s">
+      <c r="E14" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="F14" s="14" t="s">
+      <c r="F14" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="G14" s="11" t="s">
+      <c r="G14" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="H14" s="11" t="n">
+      <c r="H14" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="I14" s="15" t="s">
+      <c r="I14" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="16" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="16" t="s">
+      <c r="A15" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="C15" s="20" t="s">
+      <c r="C15" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="D15" s="17" t="s">
+      <c r="D15" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="18" t="s">
+      <c r="E15" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="F15" s="18" t="s">
+      <c r="F15" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="G15" s="16" t="s">
+      <c r="G15" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="H15" s="16" t="n">
+      <c r="H15" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="I15" s="15" t="s">
+      <c r="I15" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="n">
+      <c r="A16" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="C16" s="21" t="s">
+      <c r="C16" s="22" t="s">
         <v>72</v>
       </c>
-      <c r="D16" s="13" t="s">
+      <c r="D16" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="E16" s="14" t="s">
+      <c r="E16" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="F16" s="14" t="s">
+      <c r="F16" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="G16" s="11" t="s">
+      <c r="G16" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="H16" s="11" t="n">
+      <c r="H16" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="I16" s="15" t="s">
+      <c r="I16" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="16" t="n">
+      <c r="A17" s="17" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="16" t="s">
+      <c r="B17" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="C17" s="21" t="s">
+      <c r="C17" s="22" t="s">
         <v>72</v>
       </c>
-      <c r="D17" s="17" t="s">
+      <c r="D17" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="E17" s="18" t="s">
+      <c r="E17" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="F17" s="18" t="s">
+      <c r="F17" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="G17" s="16" t="s">
+      <c r="G17" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="H17" s="16" t="n">
+      <c r="H17" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="I17" s="15" t="s">
+      <c r="I17" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="n">
+      <c r="A18" s="12" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="C18" s="22" t="s">
+      <c r="C18" s="23" t="s">
         <v>79</v>
       </c>
-      <c r="D18" s="13" t="s">
+      <c r="D18" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="E18" s="14" t="s">
+      <c r="E18" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="F18" s="14" t="s">
+      <c r="F18" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="G18" s="11" t="s">
+      <c r="G18" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="H18" s="11" t="n">
+      <c r="H18" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="I18" s="15" t="s">
+      <c r="I18" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="16" t="n">
+      <c r="A19" s="17" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="16" t="s">
+      <c r="B19" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="C19" s="22" t="s">
+      <c r="C19" s="23" t="s">
         <v>79</v>
       </c>
-      <c r="D19" s="17" t="s">
+      <c r="D19" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="E19" s="18" t="s">
+      <c r="E19" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="F19" s="18" t="s">
+      <c r="F19" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="G19" s="16" t="s">
+      <c r="G19" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="H19" s="16" t="n">
+      <c r="H19" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="I19" s="15" t="s">
+      <c r="I19" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="n">
+      <c r="A20" s="12" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="C20" s="22" t="s">
+      <c r="C20" s="23" t="s">
         <v>79</v>
       </c>
-      <c r="D20" s="13" t="s">
+      <c r="D20" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="E20" s="14" t="s">
+      <c r="E20" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="F20" s="14" t="s">
+      <c r="F20" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="G20" s="11" t="s">
+      <c r="G20" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="H20" s="11" t="n">
+      <c r="H20" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="I20" s="15" t="s">
+      <c r="I20" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="16" t="n">
+      <c r="A21" s="17" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="16" t="s">
+      <c r="B21" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="C21" s="23" t="s">
+      <c r="C21" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="D21" s="17" t="s">
+      <c r="D21" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="E21" s="18" t="s">
+      <c r="E21" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="F21" s="18" t="s">
+      <c r="F21" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="G21" s="16" t="s">
+      <c r="G21" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="H21" s="16" t="n">
+      <c r="H21" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="I21" s="15" t="s">
+      <c r="I21" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11" t="n">
+      <c r="A22" s="12" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="C22" s="23" t="s">
+      <c r="C22" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="D22" s="13" t="s">
+      <c r="D22" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="E22" s="14" t="s">
+      <c r="E22" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="F22" s="14" t="s">
+      <c r="F22" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="G22" s="11" t="s">
+      <c r="G22" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="H22" s="11" t="n">
+      <c r="H22" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="I22" s="15" t="s">
+      <c r="I22" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="16" t="n">
+      <c r="A23" s="17" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="16" t="s">
+      <c r="B23" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="C23" s="23" t="s">
+      <c r="C23" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="D23" s="17" t="s">
+      <c r="D23" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="E23" s="18" t="s">
+      <c r="E23" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="F23" s="18" t="s">
+      <c r="F23" s="19" t="s">
         <v>98</v>
       </c>
-      <c r="G23" s="16" t="s">
+      <c r="G23" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="H23" s="16" t="n">
+      <c r="H23" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="I23" s="15" t="s">
+      <c r="I23" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="11" t="n">
+      <c r="A24" s="12" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="11" t="s">
+      <c r="B24" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="C24" s="23" t="s">
+      <c r="C24" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="D24" s="13" t="s">
+      <c r="D24" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="E24" s="14" t="s">
+      <c r="E24" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="F24" s="14" t="s">
+      <c r="F24" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="G24" s="11" t="s">
+      <c r="G24" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="H24" s="11" t="n">
+      <c r="H24" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="I24" s="15" t="s">
+      <c r="I24" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="16" t="n">
+      <c r="A25" s="17" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="16" t="s">
+      <c r="B25" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="C25" s="23" t="s">
+      <c r="C25" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="D25" s="17" t="s">
+      <c r="D25" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="E25" s="18" t="s">
+      <c r="E25" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="F25" s="18" t="s">
+      <c r="F25" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="G25" s="16" t="s">
+      <c r="G25" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="H25" s="16" t="n">
+      <c r="H25" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="I25" s="15" t="s">
+      <c r="I25" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="11" t="n">
+      <c r="A26" s="12" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="11" t="s">
+      <c r="B26" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="C26" s="23" t="s">
+      <c r="C26" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="D26" s="13" t="s">
+      <c r="D26" s="14" t="s">
         <v>96</v>
       </c>
-      <c r="E26" s="14" t="s">
+      <c r="E26" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="F26" s="14" t="s">
+      <c r="F26" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="G26" s="11" t="s">
+      <c r="G26" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="H26" s="11" t="n">
+      <c r="H26" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="I26" s="15" t="s">
+      <c r="I26" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="16" t="n">
+      <c r="A27" s="17" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="16" t="s">
+      <c r="B27" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="C27" s="23" t="s">
+      <c r="C27" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="D27" s="17" t="s">
+      <c r="D27" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="E27" s="18" t="s">
+      <c r="E27" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="F27" s="18" t="s">
+      <c r="F27" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="G27" s="16" t="s">
+      <c r="G27" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="H27" s="16" t="n">
+      <c r="H27" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="I27" s="15" t="s">
+      <c r="I27" s="16" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1896,123 +1900,123 @@
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="25" t="s">
         <v>110</v>
       </c>
-      <c r="C1" s="24" t="s">
+      <c r="C1" s="25" t="s">
         <v>111</v>
       </c>
-      <c r="D1" s="24" t="s">
+      <c r="D1" s="25" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="25" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="26" t="n">
+      <c r="B2" s="27" t="n">
         <f aca="false">COUNTIF(Planning!$D$2:$D$27,A2)</f>
         <v>11</v>
       </c>
-      <c r="C2" s="26" t="n">
+      <c r="C2" s="27" t="n">
         <f aca="false">SUMIF(Planning!$D$2:$D$27,A2,Planning!$H$2:$H$27)</f>
         <v>14.5</v>
       </c>
-      <c r="D2" s="26" t="n">
+      <c r="D2" s="27" t="n">
         <f aca="false">COUNTIFS(Planning!$D$2:$D$27,A2,Planning!$I$2:$I$27,"Terminé")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="27" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="28" t="n">
+      <c r="B3" s="29" t="n">
         <f aca="false">COUNTIF(Planning!$D$2:$D$27,A3)</f>
         <v>4</v>
       </c>
-      <c r="C3" s="28" t="n">
+      <c r="C3" s="29" t="n">
         <f aca="false">SUMIF(Planning!$D$2:$D$27,A3,Planning!$H$2:$H$27)</f>
         <v>7</v>
       </c>
-      <c r="D3" s="28" t="n">
+      <c r="D3" s="29" t="n">
         <f aca="false">COUNTIFS(Planning!$D$2:$D$27,A3,Planning!$I$2:$I$27,"Terminé")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="25" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="26" t="n">
+      <c r="B4" s="27" t="n">
         <f aca="false">COUNTIF(Planning!$D$2:$D$27,A4)</f>
         <v>5</v>
       </c>
-      <c r="C4" s="26" t="n">
+      <c r="C4" s="27" t="n">
         <f aca="false">SUMIF(Planning!$D$2:$D$27,A4,Planning!$H$2:$H$27)</f>
         <v>7</v>
       </c>
-      <c r="D4" s="26" t="n">
+      <c r="D4" s="27" t="n">
         <f aca="false">COUNTIFS(Planning!$D$2:$D$27,A4,Planning!$I$2:$I$27,"Terminé")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="27" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="28" t="n">
+      <c r="B5" s="29" t="n">
         <f aca="false">COUNTIF(Planning!$D$2:$D$27,A5)</f>
         <v>4</v>
       </c>
-      <c r="C5" s="28" t="n">
+      <c r="C5" s="29" t="n">
         <f aca="false">SUMIF(Planning!$D$2:$D$27,A5,Planning!$H$2:$H$27)</f>
         <v>6</v>
       </c>
-      <c r="D5" s="28" t="n">
+      <c r="D5" s="29" t="n">
         <f aca="false">COUNTIFS(Planning!$D$2:$D$27,A5,Planning!$I$2:$I$27,"Terminé")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="25" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="26" t="s">
         <v>96</v>
       </c>
-      <c r="B6" s="26" t="n">
+      <c r="B6" s="27" t="n">
         <f aca="false">COUNTIF(Planning!$D$2:$D$27,A6)</f>
         <v>2</v>
       </c>
-      <c r="C6" s="26" t="n">
+      <c r="C6" s="27" t="n">
         <f aca="false">SUMIF(Planning!$D$2:$D$27,A6,Planning!$H$2:$H$27)</f>
         <v>3</v>
       </c>
-      <c r="D6" s="26" t="n">
+      <c r="D6" s="27" t="n">
         <f aca="false">COUNTIFS(Planning!$D$2:$D$27,A6,Planning!$I$2:$I$27,"Terminé")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="29" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="30" t="s">
         <v>113</v>
       </c>
-      <c r="B7" s="30" t="n">
+      <c r="B7" s="31" t="n">
         <f aca="false">SUM(B2:B6)</f>
         <v>26</v>
       </c>
-      <c r="C7" s="30" t="n">
+      <c r="C7" s="31" t="n">
         <f aca="false">SUM(C2:C6)</f>
         <v>37.5</v>
       </c>
-      <c r="D7" s="30" t="n">
+      <c r="D7" s="31" t="n">
         <f aca="false">SUM(D2:D6)</f>
         <v>0</v>
       </c>

</xml_diff>